<commit_message>
chore: sync Nova upm-release-2026.08.06-01
</commit_message>
<xml_diff>
--- a/Assets/Samples/GameBindDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
+++ b/Assets/Samples/GameBindDemo/Excels/Networks/Cmds/NetworkCmds.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="12660"/>
+    <workbookView windowHeight="16660"/>
   </bookViews>
   <sheets>
     <sheet name="NetworkCmds" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
   <si>
     <t>##comment</t>
   </si>
@@ -125,6 +125,15 @@
     <t>/v1/account/bind/resolve</t>
   </si>
   <si>
+    <t>GameAccountBindingQuery</t>
+  </si>
+  <si>
+    <t>绑定查询</t>
+  </si>
+  <si>
+    <t>/v1/account/openid-bound</t>
+  </si>
+  <si>
     <t>GameSaveGet</t>
   </si>
   <si>
@@ -153,6 +162,15 @@
   </si>
   <si>
     <t>TGAServer</t>
+  </si>
+  <si>
+    <t>AppCustomConfig</t>
+  </si>
+  <si>
+    <t>拉取GM后台应用配置URL</t>
+  </si>
+  <si>
+    <t>/v1/common/app-config</t>
   </si>
 </sst>
 </file>
@@ -1208,9 +1226,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U48"/>
+  <dimension ref="A1:U49"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -1468,38 +1486,38 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
     </row>
-    <row r="10" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8" t="s">
+    <row r="10" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A10" s="1"/>
+      <c r="B10" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="3"/>
     </row>
     <row r="11" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
       <c r="A11" s="7"/>
@@ -1543,12 +1561,14 @@
         <v>39</v>
       </c>
       <c r="D12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="8"/>
@@ -1565,34 +1585,54 @@
       <c r="T12" s="8"/>
       <c r="U12" s="8"/>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>AppCustomConfig</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>拉取GM后台应用配置URL</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>HTTP_POST</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>GameServer</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>/v1/common/app-config</t>
-        </is>
-      </c>
+    <row r="13" s="2" customFormat="1" ht="22" customHeight="1" spans="1:21">
+      <c r="A13" s="7"/>
+      <c r="B13" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
     </row>
-    <row r="14" ht="22" customHeight="1"/>
+    <row r="14" ht="22" customHeight="1" spans="1:21">
+      <c r="B14" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1"/>
     <row r="17" ht="22" customHeight="1"/>
@@ -1627,6 +1667,7 @@
     <row r="46" ht="22" customHeight="1"/>
     <row r="47" ht="22" customHeight="1"/>
     <row r="48" ht="22" customHeight="1"/>
+    <row r="49" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>